<commit_message>
Fixed security, locking and resource leaking (in session) bugs
</commit_message>
<xml_diff>
--- a/examples/workbook.xlsx
+++ b/examples/workbook.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,7 +682,7 @@
         <v>25.5</v>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -709,6 +709,23 @@
       </c>
       <c r="C5" t="n">
         <v>50</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Car Part</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>99.00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>